<commit_message>
Pivot métier : nettoyage automobile remplacé par nettoyage de bureaux
- Nouvelle page /nettoyage-bureaux/ (contenu complet : entretien, déroulé,
  prix, 6 FAQ autoportantes, schema Service/Breadcrumb/FAQPage), /nettoyage-automobile/ supprimée
- Nouvelle photo Pexels 6197108 (équipe en intervention, jamais utilisée) en 600/900/1200w
- Accueil : title/meta/OG, carte 03, kicker, manifeste, protocole, trust,
  avis (Laurent office manager), FAQ, schema (description, knowsAbout, OfferCatalog)
- Selects de formulaire, footers, sitemap, llms.txt, README, xlsx de suivi : tout basculé
- Zéro trace automobile/véhicule restante (grep vérifié), 5 pages schemas valides, liens 200

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/suivi-leads-klynera.xlsx
+++ b/tracking/suivi-leads-klynera.xlsx
@@ -5627,6 +5627,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -5728,7 +5729,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Nettoyage automobile</t>
+          <t>Nettoyage de bureaux</t>
         </is>
       </c>
       <c r="E8" s="4">
@@ -5825,6 +5826,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>

</xml_diff>